<commit_message>
Stage 8 review fixes: G-007
</commit_message>
<xml_diff>
--- a/output/heldback_firm_G/OsterquillData/Studies/OT-08-S0114/Raw_Observations/AP02_Genotox_RAW_111708.xlsx
+++ b/output/heldback_firm_G/OsterquillData/Studies/OT-08-S0114/Raw_Observations/AP02_Genotox_RAW_111708.xlsx
@@ -167,36 +167,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Kenji Morita</author>
-  </authors>
-  <commentList>
-    <comment ref="B7" authorId="0" shapeId="0">
-      <text>
-        <t>Outcome text not yet agreed with Avernelwick. Hold the summary until the mammalian sheet is signed off.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Lucia Moretti</author>
-  </authors>
-  <commentList>
-    <comment ref="A4" authorId="0" shapeId="0">
-      <text>
-        <t>Mammalian signal does not line up with the Ames plates. Discuss at the next QA gate before Avernelwick sees the sheet.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -530,7 +500,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>OT-08-S0114 observation sheets: AP02 genotoxicity battery</t>
+          <t>Osterquill Toxicology Inc | OT-08-S0114 observation sheets: AP02 genotoxicity battery</t>
         </is>
       </c>
     </row>
@@ -618,7 +588,7 @@
       <c r="C8" s="2" t="n"/>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Checked by Lucia Moretti 11/03/2008</t>
+          <t>Prepared by Kenji Morita; QA and approval records retained separately</t>
         </is>
       </c>
     </row>
@@ -728,7 +698,6 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1127,7 +1096,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Control validity: each strain's positive control is recorded on the bench sheet, not repeated here.</t>
+          <t>Control validity: positive-control responses and acceptance decisions are not tabulated here; consult the original investigation records before interpreting the outcome.</t>
         </is>
       </c>
     </row>
@@ -2898,14 +2867,14 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Mammalian-cell micronucleus assessment (TK6). Treatment 3 h with and without S9, recovery to 24 h. Percent micronucleated cells, RPD against vehicle.</t>
+          <t>Mammalian-cell micronucleus assessment (TK6). Treatments: 3 h with S9, 3 h without S9 and 24 h without S9. Percent micronucleated cells; relative population doubling (RPD) against matched vehicle.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Scoring on each culture by two readers, blind to treatment. Discordant reads are re-scored by the study director.</t>
+          <t>Displayed frequencies do not show a consistent concentration-related increase over matched vehicles. Article attribution and control acceptance must be checked in the investigation records before interpretation.</t>
         </is>
       </c>
     </row>
@@ -3141,6 +3110,5 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>